<commit_message>
feat: Implement automatic synchronization of account statements for each server upon finalizing the official document
- Added a summary section in the official document wizard to display account statements for each server.
- Updated the list view for account statements to indicate that they are created automatically from finalized documents.
- Enhanced the account statement creation process to ensure one statement per server.
- Introduced autosave functionality in the account statement forms to improve user experience.
- Created tests to verify the automatic creation and synchronization of account statements.
- Refactored JavaScript for autosave functionality to handle form submissions and field updates efficiently.
</commit_message>
<xml_diff>
--- a/documentos/templates_xlsx/diario_bordo/modelo_diario_bordo.xlsx
+++ b/documentos/templates_xlsx/diario_bordo/modelo_diario_bordo.xlsx
@@ -123,6 +123,7 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font/>
     <font>
       <b/>
       <sz val="11.0"/>
@@ -130,7 +131,6 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
-    <font/>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
@@ -145,48 +145,130 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="25">
     <border/>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+        <color rgb="FFFFFFFF"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
     </border>
     <border>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFFFFFFF"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+        <color rgb="FFFFFFFF"/>
+      </top>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFFFFFFF"/>
+      </left>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFFFFFFF"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
+        <color rgb="FFFFFFFF"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -214,17 +296,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -269,65 +340,64 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="14" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="15" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="18" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="19" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="20" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="18" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="13" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="13" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="12" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="13" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="21" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="22" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="23" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="24" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -340,8 +410,8 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>876300</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>942975</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -575,236 +645,334 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="10" width="17.0"/>
+    <col customWidth="1" min="1" max="12" width="18.13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1">
       <c r="A1" s="1"/>
-    </row>
-    <row r="2" ht="20.25" customHeight="1"/>
-    <row r="3" ht="20.25" customHeight="1"/>
-    <row r="4" ht="20.25" customHeight="1"/>
-    <row r="5" ht="20.25" customHeight="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="3"/>
+    </row>
+    <row r="2" ht="20.25" customHeight="1">
+      <c r="A2" s="4"/>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" ht="20.25" customHeight="1">
+      <c r="A3" s="4"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" ht="20.25" customHeight="1">
+      <c r="A4" s="4"/>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" ht="20.25" customHeight="1">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="8"/>
+    </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="9" t="s">
         <v>0</v>
       </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="11"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="9" t="s">
         <v>1</v>
       </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="11"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="9" t="s">
         <v>2</v>
       </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="11"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="11"/>
     </row>
     <row r="10" ht="7.5" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" ht="24.75" customHeight="1">
-      <c r="A11" s="4" t="s">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+    </row>
+    <row r="11" ht="30.75" customHeight="1">
+      <c r="A11" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="4" t="s">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" ht="24.75" customHeight="1">
-      <c r="A12" s="4" t="s">
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="15"/>
+    </row>
+    <row r="12" ht="30.75" customHeight="1">
+      <c r="A12" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="4" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" ht="24.75" customHeight="1">
-      <c r="A13" s="4" t="s">
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="15"/>
+    </row>
+    <row r="13" ht="30.75" customHeight="1">
+      <c r="A13" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="4" t="s">
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="6"/>
-    </row>
-    <row r="14" ht="24.75" customHeight="1">
-      <c r="A14" s="7"/>
-    </row>
-    <row r="15" ht="24.75" customHeight="1">
-      <c r="A15" s="8" t="s">
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="15"/>
+    </row>
+    <row r="14" ht="30.75" customHeight="1">
+      <c r="A14" s="16"/>
+      <c r="L14" s="5"/>
+    </row>
+    <row r="15" ht="30.75" customHeight="1">
+      <c r="A15" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="8" t="s">
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="9" t="s">
+      <c r="E15" s="14"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="19"/>
+      <c r="I15" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="J15" s="19"/>
+      <c r="K15" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="J15" s="11"/>
-    </row>
-    <row r="16" ht="24.75" customHeight="1">
-      <c r="A16" s="12" t="s">
+      <c r="L15" s="19"/>
+    </row>
+    <row r="16" ht="30.75" customHeight="1">
+      <c r="A16" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="15"/>
-    </row>
-    <row r="17" ht="24.75" customHeight="1">
-      <c r="A17" s="16" t="s">
+      <c r="G16" s="21"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="22"/>
+    </row>
+    <row r="17" ht="30.75" customHeight="1">
+      <c r="A17" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="15"/>
+      <c r="I17" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="20" t="s">
+      <c r="J17" s="15"/>
+      <c r="K17" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="J17" s="6"/>
+      <c r="L17" s="15"/>
     </row>
     <row r="18" ht="24.75" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="21" t="s">
+      <c r="B18" s="27"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="21" t="s">
+      <c r="E18" s="27"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="11"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="19"/>
     </row>
     <row r="19" ht="24.75" customHeight="1">
-      <c r="A19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="23"/>
-      <c r="J19" s="24"/>
+      <c r="A19" s="28"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="28"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="28"/>
+      <c r="L19" s="29"/>
     </row>
     <row r="20" ht="24.75" customHeight="1">
-      <c r="A20" s="14"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="15"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A1:J5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
+  <mergeCells count="23">
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A1:L5"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="G12:L12"/>
+    <mergeCell ref="G13:L13"/>
+    <mergeCell ref="K15:L16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="A18:C20"/>
+    <mergeCell ref="D18:F20"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="G17:H17"/>
     <mergeCell ref="I15:J16"/>
     <mergeCell ref="I17:J17"/>
-    <mergeCell ref="A18:C20"/>
-    <mergeCell ref="D18:F20"/>
-    <mergeCell ref="G18:J20"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G18:L20"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>